<commit_message>
Filter supplier order by product (burger-only support)
- supplier_order_from_sales accepts optional product_id; joins consumption_log
  through orders to scope the calculation to one product's sales only
- /supplier-order page gets a product dropdown (defaults to 'all')
- Excel gets a second sheet "הזמנה לספק - המבורגר בלבד" generated alongside
  the all-products sheet

Example (same day, 2026-04-23):
  All products : 93 mnot, revenue ₪5,664  ->  supplier order ₪2,754.50 (48.6%)
  Burger only  : 47 mnot, revenue ₪3,040  ->  supplier order ₪1,406.50 (46.3%)

https://claude.ai/code/session_01PT2i4QroDVpmnQ16J8pp1q
</commit_message>
<xml_diff>
--- a/fixi_export.xlsx
+++ b/fixi_export.xlsx
@@ -19,6 +19,7 @@
     <sheet name="תכנית שבועית" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="הזמנה יומית" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="הזמנה לספק (לפי מכירות)" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="הזמנה לספק - המבורגר בלבד" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2750,6 +2751,933 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>הזמנה לספקים לפי מכירות יום 2026-04-23 - המבורגר בלבד</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>מכירות: 47 מנות · הכנסה ₪3040.00 · עלות הזמנה לספקים: ₪1406.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>ספק</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>פריט</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>אריזה</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>צריכה במטבח</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>יחידת מטבח</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>פחת %</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>נדרש (כולל פחת)</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>כמות בחבילה</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>מס' חבילות להזמין</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>כמות בפועל שמגיעה</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>עודף (מעבר לנדרש)</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>מחיר חבילה</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>סה"כ לפריט</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>מאפיית הבוקר</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>לחמניית המבורגר</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ארגז 30 יחידות</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>47</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>47.96</v>
+      </c>
+      <c r="H5" t="n">
+        <v>30</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" t="n">
+        <v>60</v>
+      </c>
+      <c r="K5" t="n">
+        <v>12.04</v>
+      </c>
+      <c r="L5" t="n">
+        <v>75</v>
+      </c>
+      <c r="M5" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>סה"כ מאפיית הבוקר</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="7" t="n"/>
+      <c r="J6" s="7" t="n"/>
+      <c r="K6" s="7" t="n"/>
+      <c r="L6" s="7" t="n"/>
+      <c r="M6" s="5" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>בשר איכות בע"מ</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>קציצת בקר 180 גרם</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ארגז 20 יחידות</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>47</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G7" t="n">
+        <v>48.21</v>
+      </c>
+      <c r="H7" t="n">
+        <v>20</v>
+      </c>
+      <c r="I7" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" t="n">
+        <v>60</v>
+      </c>
+      <c r="K7" t="n">
+        <v>11.79</v>
+      </c>
+      <c r="L7" t="n">
+        <v>180</v>
+      </c>
+      <c r="M7" t="n">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>סה"כ בשר איכות בע"מ</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="7" t="n"/>
+      <c r="J8" s="7" t="n"/>
+      <c r="K8" s="7" t="n"/>
+      <c r="L8" s="7" t="n"/>
+      <c r="M8" s="5" t="n">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>תנובה מוצרי חלב</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>גבינה צהובה</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>גלגל 2.5 ק"ג</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1175</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>gram</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1211.34</v>
+      </c>
+      <c r="H9" t="n">
+        <v>2500</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="n">
+        <v>2500</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1288.66</v>
+      </c>
+      <c r="L9" t="n">
+        <v>200</v>
+      </c>
+      <c r="M9" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>סה"כ תנובה מוצרי חלב</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
+      <c r="J10" s="7" t="n"/>
+      <c r="K10" s="7" t="n"/>
+      <c r="L10" s="7" t="n"/>
+      <c r="M10" s="5" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ירקות השוק</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>בצל</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>שק 10 ק"ג</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>940</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>gram</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>15</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1105.88</v>
+      </c>
+      <c r="H11" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" t="n">
+        <v>10000</v>
+      </c>
+      <c r="K11" t="n">
+        <v>8894.120000000001</v>
+      </c>
+      <c r="L11" t="n">
+        <v>100</v>
+      </c>
+      <c r="M11" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ירקות השוק</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>עגבנייה</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ארגז 5 ק"ג</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1880</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>gram</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>8</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2043.48</v>
+      </c>
+      <c r="H12" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" t="n">
+        <v>5000</v>
+      </c>
+      <c r="K12" t="n">
+        <v>2956.52</v>
+      </c>
+      <c r="L12" t="n">
+        <v>75</v>
+      </c>
+      <c r="M12" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ירקות השוק</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>חסה</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ראש 300 גרם</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>940</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>gram</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>12</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1068.18</v>
+      </c>
+      <c r="H13" t="n">
+        <v>300</v>
+      </c>
+      <c r="I13" t="n">
+        <v>4</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1200</v>
+      </c>
+      <c r="K13" t="n">
+        <v>131.82</v>
+      </c>
+      <c r="L13" t="n">
+        <v>6</v>
+      </c>
+      <c r="M13" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>סה"כ ירקות השוק</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="7" t="n"/>
+      <c r="J14" s="7" t="n"/>
+      <c r="K14" s="7" t="n"/>
+      <c r="L14" s="7" t="n"/>
+      <c r="M14" s="5" t="n">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>חומץ מעדנות</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>מלפפון חמוץ</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>קופסה 2.5 ק"ג</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>705</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>gram</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" t="n">
+        <v>726.8</v>
+      </c>
+      <c r="H15" t="n">
+        <v>2500</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" t="n">
+        <v>2500</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1773.2</v>
+      </c>
+      <c r="L15" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="M15" t="n">
+        <v>62.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>סה"כ חומץ מעדנות</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
+      <c r="J16" s="7" t="n"/>
+      <c r="K16" s="7" t="n"/>
+      <c r="L16" s="7" t="n"/>
+      <c r="M16" s="5" t="n">
+        <v>62.5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>רטבי היום</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>רוטב המבורגר</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>קופסה 1 ליטר</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1410</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1453.61</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I17" t="n">
+        <v>2</v>
+      </c>
+      <c r="J17" t="n">
+        <v>2000</v>
+      </c>
+      <c r="K17" t="n">
+        <v>546.39</v>
+      </c>
+      <c r="L17" t="n">
+        <v>30</v>
+      </c>
+      <c r="M17" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>סה"כ רטבי היום</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="7" t="n"/>
+      <c r="I18" s="7" t="n"/>
+      <c r="J18" s="7" t="n"/>
+      <c r="K18" s="7" t="n"/>
+      <c r="L18" s="7" t="n"/>
+      <c r="M18" s="5" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>אריזות השולחן</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>קופסת המבורגר קרטון</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ארגז 100 יחידות</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>21</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G19" t="n">
+        <v>21.32</v>
+      </c>
+      <c r="H19" t="n">
+        <v>100</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" t="n">
+        <v>100</v>
+      </c>
+      <c r="K19" t="n">
+        <v>78.68000000000001</v>
+      </c>
+      <c r="L19" t="n">
+        <v>120</v>
+      </c>
+      <c r="M19" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>אריזות השולחן</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>שקית נייר ניידים</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>חבילה 50 יחידות</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>21</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="n">
+        <v>21.21</v>
+      </c>
+      <c r="H20" t="n">
+        <v>50</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" t="n">
+        <v>50</v>
+      </c>
+      <c r="K20" t="n">
+        <v>28.79</v>
+      </c>
+      <c r="L20" t="n">
+        <v>35</v>
+      </c>
+      <c r="M20" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>סה"כ אריזות השולחן</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n"/>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="n"/>
+      <c r="H21" s="7" t="n"/>
+      <c r="I21" s="7" t="n"/>
+      <c r="J21" s="7" t="n"/>
+      <c r="K21" s="7" t="n"/>
+      <c r="L21" s="7" t="n"/>
+      <c r="M21" s="5" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>כלי חד פעמי טל</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>מזלג חד פעמי</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>חבילה 100 יחידות</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>21</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G22" t="n">
+        <v>21.11</v>
+      </c>
+      <c r="H22" t="n">
+        <v>100</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" t="n">
+        <v>100</v>
+      </c>
+      <c r="K22" t="n">
+        <v>78.89</v>
+      </c>
+      <c r="L22" t="n">
+        <v>15</v>
+      </c>
+      <c r="M22" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>כלי חד פעמי טל</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>סכין חד פעמי</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>חבילה 100 יחידות</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>21</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G23" t="n">
+        <v>21.11</v>
+      </c>
+      <c r="H23" t="n">
+        <v>100</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" t="n">
+        <v>100</v>
+      </c>
+      <c r="K23" t="n">
+        <v>78.89</v>
+      </c>
+      <c r="L23" t="n">
+        <v>15</v>
+      </c>
+      <c r="M23" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>כלי חד פעמי טל</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>מפית נייר</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>חבילה 200 יחידות</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>94</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="n">
+        <v>94.95</v>
+      </c>
+      <c r="H24" t="n">
+        <v>200</v>
+      </c>
+      <c r="I24" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" t="n">
+        <v>200</v>
+      </c>
+      <c r="K24" t="n">
+        <v>105.05</v>
+      </c>
+      <c r="L24" t="n">
+        <v>10</v>
+      </c>
+      <c r="M24" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>סה"כ כלי חד פעמי טל</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n"/>
+      <c r="C25" s="7" t="n"/>
+      <c r="D25" s="7" t="n"/>
+      <c r="E25" s="7" t="n"/>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="n"/>
+      <c r="H25" s="7" t="n"/>
+      <c r="I25" s="7" t="n"/>
+      <c r="J25" s="7" t="n"/>
+      <c r="K25" s="7" t="n"/>
+      <c r="L25" s="7" t="n"/>
+      <c r="M25" s="5" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>סה"כ כללי</t>
+        </is>
+      </c>
+      <c r="M27" s="9" t="n">
+        <v>1406.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>